<commit_message>
Use recovery-only quote budget in downloadable models
</commit_message>
<xml_diff>
--- a/excel/templates/Flap_BSC_RWA币股_控筹模型.xlsx
+++ b/excel/templates/Flap_BSC_RWA币股_控筹模型.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="控筹模型" sheetId="1" r:id="Ree9c4e9602624388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quote参数" sheetId="2" r:id="Rff154de45f2d40ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="控筹模型" sheetId="1" r:id="Rdfcf5d9f72a04e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quote参数" sheetId="2" r:id="Rc51882bdca6f4145"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="10">
+  <x:numFmts count="11">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.000000"/>
@@ -25,6 +25,7 @@
     <x:numFmt numFmtId="207" formatCode="0.0000%"/>
     <x:numFmt numFmtId="208" formatCode="#,##0"/>
     <x:numFmt numFmtId="209" formatCode="0.0000000000"/>
+    <x:numFmt numFmtId="210" formatCode=";;;"/>
   </x:numFmts>
   <x:fonts count="12">
     <x:font>
@@ -162,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="149">
+  <x:cellXfs count="150">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -601,6 +602,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="210" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1308,8 +1312,8 @@
         <v>建议 Quote 资金</v>
       </c>
       <c r="D18" s="114" t="n">
-        <f>IF(ISNUMBER($D$26),(IF(LEFT($D$51,2)&lt;&gt;"可达","",IF($D$22="","",SUM($D$22,$D$23,$D$24,$D$25))))+$D$26,"")</f>
-        <v>572.247068230949</v>
+        <f>IF(AND(LEFT($D$51,2)="可达",ISNUMBER($D$22),ISNUMBER($D$23),ISNUMBER($D$25),ISNUMBER($D$26)),SUM($D$22:$D$23,$D$25:$D$26),"")</f>
+        <v>536.5327825179661</v>
       </c>
       <c r="E18" s="58" t="str">
         <f>$D$7</f>
@@ -1330,7 +1334,7 @@
       </c>
       <c r="J18" s="114" t="n">
         <f>IF(AND(ISNUMBER($D$19),ISNUMBER($G$19)),SUM(D19,G19),"")</f>
-        <v>88982.48906742512</v>
+        <v>83532.39978190965</v>
       </c>
       <c r="K18" s="58" t="str">
         <v>USDT</v>
@@ -1345,7 +1349,7 @@
       </c>
       <c r="D19" s="115" t="n">
         <f>IF(ISNUMBER($D$18),IF($D$18=0,0,IF($D$55&gt;0,$D$18*$D$55,"")),"")</f>
-        <v>87326.33322971339</v>
+        <v>81876.24394419792</v>
       </c>
       <c r="E19" s="100" t="str">
         <v>USDT</v>
@@ -1454,16 +1458,11 @@
       <c r="K23" s="100"/>
       <c r="L23" s="100"/>
     </row>
-    <row r="24" ht="20" customHeight="1">
+    <row r="24" customHeight="1" hidden="1">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="101" t="str">
-        <v>洗筹损耗</v>
-      </c>
-      <c r="D24" s="115" t="n">
-        <f>IF(LEFT($D$51,2)&lt;&gt;"可达","",IF($J$46="","",$J$46*$J$47))</f>
-        <v>35.71428571298285</v>
-      </c>
+      <c r="C24" s="101"/>
+      <c r="D24" s="149"/>
       <c r="E24" s="100" t="str">
         <f>$D$7</f>
         <v>SPCXB</v>
@@ -1692,7 +1691,7 @@
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="108" t="str">
-        <v>外盘一卖一买使用卖出所得 Quote 回买；洗后若低于目标，再按外盘曲线差额及买入费预留恢复所需 Quote。洗筹损耗另列；未模拟成交量、滑点与价格冲击。</v>
+        <v>外盘一卖一买使用卖出所得 Quote 回买；手续费仅降低洗后持币，不另列资金。洗后若低于目标，再按外盘曲线差额及买入费预留恢复所需 Quote；未模拟成交量、滑点与价格冲击。</v>
       </c>
       <c r="D36" s="108"/>
       <c r="E36" s="108"/>

</xml_diff>